<commit_message>
add raw xlsx file
</commit_message>
<xml_diff>
--- a/data/raw/Treasury data 090426.xlsx
+++ b/data/raw/Treasury data 090426.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\VFE\VFE 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samla\zcb_treasury_curve\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F96E55C5-C34F-4C4F-A880-F09110D39924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76CE867-73AE-4DC2-9F40-149649A0789B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{AE0A35FC-EEFE-4C79-9745-D25756466BC9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{AE0A35FC-EEFE-4C79-9745-D25756466BC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -90,7 +90,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,7 +204,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -214,10 +216,11 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,85 +556,64 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11933CD4-8E68-40CE-B532-BA56B007F1D6}">
   <dimension ref="B2:I362"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="3.6328125" customWidth="1"/>
+    <col min="2" max="2" width="10.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="17.25" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:9" ht="17.5">
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B3" s="9" t="s">
+    </row>
+    <row r="3" spans="2:9">
+      <c r="B3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-    </row>
-    <row r="4" spans="2:9" ht="17.649999999999999" x14ac:dyDescent="0.45">
-      <c r="B4" s="8" t="s">
+    </row>
+    <row r="4" spans="2:9" ht="18">
+      <c r="B4" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-    </row>
-    <row r="5" spans="2:9" ht="17.649999999999999" x14ac:dyDescent="0.45">
-      <c r="B5" s="8"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B6" s="11" t="s">
+    </row>
+    <row r="5" spans="2:9" ht="18">
+      <c r="B5" s="7"/>
+    </row>
+    <row r="6" spans="2:9">
+      <c r="B6" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B7" s="10"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B8" s="10" t="s">
+    </row>
+    <row r="7" spans="2:9">
+      <c r="B7" s="9"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+    </row>
+    <row r="8" spans="2:9">
+      <c r="B8" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:9">
       <c r="B9" s="1">
         <v>46280</v>
       </c>
@@ -654,7 +636,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:9">
       <c r="B10" s="1">
         <v>46295</v>
       </c>
@@ -674,7 +656,7 @@
         <v>3.625</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:9">
       <c r="B11" s="1">
         <v>46295</v>
       </c>
@@ -697,7 +679,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:9">
       <c r="B12" s="1">
         <v>46295</v>
       </c>
@@ -717,7 +699,7 @@
         <v>3.6030000000000002</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:9">
       <c r="B13" s="1">
         <v>46310</v>
       </c>
@@ -740,7 +722,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:9">
       <c r="B14" s="1">
         <v>46326</v>
       </c>
@@ -760,7 +742,7 @@
         <v>3.8079999999999998</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:9">
       <c r="B15" s="1">
         <v>46326</v>
       </c>
@@ -780,7 +762,7 @@
         <v>3.7549999999999999</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:9">
       <c r="B16" s="1">
         <v>46326</v>
       </c>
@@ -800,7 +782,7 @@
         <v>3.8769999999999998</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:7">
       <c r="B17" s="1">
         <v>46341</v>
       </c>
@@ -820,7 +802,7 @@
         <v>3.7869999999999999</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:7">
       <c r="B18" s="1">
         <v>46341</v>
       </c>
@@ -840,7 +822,7 @@
         <v>3.7410000000000001</v>
       </c>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:7">
       <c r="B19" s="1">
         <v>46341</v>
       </c>
@@ -860,7 +842,7 @@
         <v>4.0579999999999998</v>
       </c>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:7">
       <c r="B20" s="1">
         <v>46356</v>
       </c>
@@ -880,7 +862,7 @@
         <v>3.7930000000000001</v>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:7">
       <c r="B21" s="1">
         <v>46356</v>
       </c>
@@ -900,7 +882,7 @@
         <v>3.7469999999999999</v>
       </c>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:7">
       <c r="B22" s="1">
         <v>46356</v>
       </c>
@@ -920,7 +902,7 @@
         <v>3.774</v>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:7">
       <c r="B23" s="1">
         <v>46371</v>
       </c>
@@ -940,7 +922,7 @@
         <v>3.7050000000000001</v>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:7">
       <c r="B24" s="1">
         <v>46387</v>
       </c>
@@ -960,7 +942,7 @@
         <v>3.8839999999999999</v>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:7">
       <c r="B25" s="1">
         <v>46387</v>
       </c>
@@ -980,7 +962,7 @@
         <v>3.8690000000000002</v>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:7">
       <c r="B26" s="1">
         <v>46387</v>
       </c>
@@ -1000,7 +982,7 @@
         <v>3.8759999999999999</v>
       </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:7">
       <c r="B27" s="1">
         <v>46402</v>
       </c>
@@ -1020,7 +1002,7 @@
         <v>3.8069999999999999</v>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:7">
       <c r="B28" s="1">
         <v>46418</v>
       </c>
@@ -1040,7 +1022,7 @@
         <v>3.9590000000000001</v>
       </c>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:7">
       <c r="B29" s="1">
         <v>46418</v>
       </c>
@@ -1060,7 +1042,7 @@
         <v>3.9550000000000001</v>
       </c>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:7">
       <c r="B30" s="1">
         <v>46433</v>
       </c>
@@ -1080,7 +1062,7 @@
         <v>3.9119999999999999</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:7">
       <c r="B31" s="1">
         <v>46433</v>
       </c>
@@ -1100,7 +1082,7 @@
         <v>3.9550000000000001</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:7">
       <c r="B32" s="1">
         <v>46433</v>
       </c>
@@ -1120,7 +1102,7 @@
         <v>3.9809999999999999</v>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:7">
       <c r="B33" s="1">
         <v>46446</v>
       </c>
@@ -1140,7 +1122,7 @@
         <v>3.9740000000000002</v>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:7">
       <c r="B34" s="1">
         <v>46446</v>
       </c>
@@ -1160,7 +1142,7 @@
         <v>3.923</v>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:7">
       <c r="B35" s="1">
         <v>46446</v>
       </c>
@@ -1180,7 +1162,7 @@
         <v>3.94</v>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:7">
       <c r="B36" s="1">
         <v>46461</v>
       </c>
@@ -1200,7 +1182,7 @@
         <v>3.9260000000000002</v>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:7">
       <c r="B37" s="1">
         <v>46477</v>
       </c>
@@ -1220,7 +1202,7 @@
         <v>3.9710000000000001</v>
       </c>
     </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:7">
       <c r="B38" s="1">
         <v>46477</v>
       </c>
@@ -1240,7 +1222,7 @@
         <v>3.964</v>
       </c>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:7">
       <c r="B39" s="1">
         <v>46477</v>
       </c>
@@ -1260,7 +1242,7 @@
         <v>3.9569999999999999</v>
       </c>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:7">
       <c r="B40" s="1">
         <v>46492</v>
       </c>
@@ -1280,7 +1262,7 @@
         <v>4.0019999999999998</v>
       </c>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:7">
       <c r="B41" s="1">
         <v>46507</v>
       </c>
@@ -1300,7 +1282,7 @@
         <v>4.024</v>
       </c>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:7">
       <c r="B42" s="1">
         <v>46507</v>
       </c>
@@ -1320,7 +1302,7 @@
         <v>4.0609999999999999</v>
       </c>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="2:7">
       <c r="B43" s="1">
         <v>46507</v>
       </c>
@@ -1340,7 +1322,7 @@
         <v>4.0170000000000003</v>
       </c>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="2:7">
       <c r="B44" s="1">
         <v>46522</v>
       </c>
@@ -1360,7 +1342,7 @@
         <v>4.0890000000000004</v>
       </c>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="2:7">
       <c r="B45" s="1">
         <v>46522</v>
       </c>
@@ -1380,7 +1362,7 @@
         <v>4.0949999999999998</v>
       </c>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:7">
       <c r="B46" s="1">
         <v>46538</v>
       </c>
@@ -1400,7 +1382,7 @@
         <v>4.069</v>
       </c>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="47" spans="2:7">
       <c r="B47" s="1">
         <v>46538</v>
       </c>
@@ -1420,7 +1402,7 @@
         <v>4.0640000000000001</v>
       </c>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="2:7">
       <c r="B48" s="1">
         <v>46538</v>
       </c>
@@ -1440,7 +1422,7 @@
         <v>4.0780000000000003</v>
       </c>
     </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="2:7">
       <c r="B49" s="1">
         <v>46553</v>
       </c>
@@ -1460,7 +1442,7 @@
         <v>4.0949999999999998</v>
       </c>
     </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="2:7">
       <c r="B50" s="1">
         <v>46568</v>
       </c>
@@ -1480,7 +1462,7 @@
         <v>4.1260000000000003</v>
       </c>
     </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="2:7">
       <c r="B51" s="1">
         <v>46568</v>
       </c>
@@ -1500,7 +1482,7 @@
         <v>4.1070000000000002</v>
       </c>
     </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="52" spans="2:7">
       <c r="B52" s="1">
         <v>46568</v>
       </c>
@@ -1520,7 +1502,7 @@
         <v>4.1310000000000002</v>
       </c>
     </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="2:7">
       <c r="B53" s="1">
         <v>46583</v>
       </c>
@@ -1540,7 +1522,7 @@
         <v>4.1429999999999998</v>
       </c>
     </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="54" spans="2:7">
       <c r="B54" s="1">
         <v>46599</v>
       </c>
@@ -1560,7 +1542,7 @@
         <v>4.17</v>
       </c>
     </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="2:7">
       <c r="B55" s="1">
         <v>46599</v>
       </c>
@@ -1580,7 +1562,7 @@
         <v>4.1769999999999996</v>
       </c>
     </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="2:7">
       <c r="B56" s="1">
         <v>46599</v>
       </c>
@@ -1600,7 +1582,7 @@
         <v>4.1680000000000001</v>
       </c>
     </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="2:7">
       <c r="B57" s="1">
         <v>46614</v>
       </c>
@@ -1620,7 +1602,7 @@
         <v>4.1680000000000001</v>
       </c>
     </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="2:7">
       <c r="B58" s="1">
         <v>46614</v>
       </c>
@@ -1640,7 +1622,7 @@
         <v>4.1689999999999996</v>
       </c>
     </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="2:7">
       <c r="B59" s="1">
         <v>46614</v>
       </c>
@@ -1660,7 +1642,7 @@
         <v>4.21</v>
       </c>
     </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="2:7">
       <c r="B60" s="1">
         <v>46630</v>
       </c>
@@ -1680,7 +1662,7 @@
         <v>4.2069999999999999</v>
       </c>
     </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="2:7">
       <c r="B61" s="1">
         <v>46630</v>
       </c>
@@ -1700,7 +1682,7 @@
         <v>4.1950000000000003</v>
       </c>
     </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="2:7">
       <c r="B62" s="1">
         <v>46630</v>
       </c>
@@ -1720,7 +1702,7 @@
         <v>4.1929999999999996</v>
       </c>
     </row>
-    <row r="63" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="2:7">
       <c r="B63" s="1">
         <v>46645</v>
       </c>
@@ -1740,7 +1722,7 @@
         <v>4.181</v>
       </c>
     </row>
-    <row r="64" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="2:7">
       <c r="B64" s="1">
         <v>46660</v>
       </c>
@@ -1760,7 +1742,7 @@
         <v>4.2039999999999997</v>
       </c>
     </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="65" spans="2:7">
       <c r="B65" s="1">
         <v>46660</v>
       </c>
@@ -1780,7 +1762,7 @@
         <v>4.2060000000000004</v>
       </c>
     </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="66" spans="2:7">
       <c r="B66" s="1">
         <v>46660</v>
       </c>
@@ -1800,7 +1782,7 @@
         <v>4.1989999999999998</v>
       </c>
     </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="67" spans="2:7">
       <c r="B67" s="1">
         <v>46675</v>
       </c>
@@ -1820,7 +1802,7 @@
         <v>4.2309999999999999</v>
       </c>
     </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="68" spans="2:7">
       <c r="B68" s="1">
         <v>46691</v>
       </c>
@@ -1840,7 +1822,7 @@
         <v>4.26</v>
       </c>
     </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="69" spans="2:7">
       <c r="B69" s="1">
         <v>46691</v>
       </c>
@@ -1860,7 +1842,7 @@
         <v>4.2460000000000004</v>
       </c>
     </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="70" spans="2:7">
       <c r="B70" s="1">
         <v>46691</v>
       </c>
@@ -1880,7 +1862,7 @@
         <v>4.2480000000000002</v>
       </c>
     </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="71" spans="2:7">
       <c r="B71" s="1">
         <v>46706</v>
       </c>
@@ -1900,7 +1882,7 @@
         <v>4.2629999999999999</v>
       </c>
     </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="72" spans="2:7">
       <c r="B72" s="1">
         <v>46706</v>
       </c>
@@ -1920,7 +1902,7 @@
         <v>4.2569999999999997</v>
       </c>
     </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="73" spans="2:7">
       <c r="B73" s="1">
         <v>46706</v>
       </c>
@@ -1940,7 +1922,7 @@
         <v>4.2670000000000003</v>
       </c>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="74" spans="2:7">
       <c r="B74" s="1">
         <v>46721</v>
       </c>
@@ -1960,7 +1942,7 @@
         <v>4.2629999999999999</v>
       </c>
     </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="75" spans="2:7">
       <c r="B75" s="1">
         <v>46721</v>
       </c>
@@ -1980,7 +1962,7 @@
         <v>4.2690000000000001</v>
       </c>
     </row>
-    <row r="76" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="76" spans="2:7">
       <c r="B76" s="1">
         <v>46721</v>
       </c>
@@ -2000,7 +1982,7 @@
         <v>4.2670000000000003</v>
       </c>
     </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="77" spans="2:7">
       <c r="B77" s="1">
         <v>46736</v>
       </c>
@@ -2020,7 +2002,7 @@
         <v>4.2770000000000001</v>
       </c>
     </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="78" spans="2:7">
       <c r="B78" s="1">
         <v>46752</v>
       </c>
@@ -2040,7 +2022,7 @@
         <v>4.2869999999999999</v>
       </c>
     </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="79" spans="2:7">
       <c r="B79" s="1">
         <v>46752</v>
       </c>
@@ -2060,7 +2042,7 @@
         <v>4.2889999999999997</v>
       </c>
     </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="80" spans="2:7">
       <c r="B80" s="1">
         <v>46752</v>
       </c>
@@ -2080,7 +2062,7 @@
         <v>4.2930000000000001</v>
       </c>
     </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="81" spans="2:7">
       <c r="B81" s="1">
         <v>46767</v>
       </c>
@@ -2100,7 +2082,7 @@
         <v>4.3070000000000004</v>
       </c>
     </row>
-    <row r="82" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="82" spans="2:7">
       <c r="B82" s="1">
         <v>46783</v>
       </c>
@@ -2120,7 +2102,7 @@
         <v>4.3079999999999998</v>
       </c>
     </row>
-    <row r="83" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="83" spans="2:7">
       <c r="B83" s="1">
         <v>46783</v>
       </c>
@@ -2140,7 +2122,7 @@
         <v>4.3029999999999999</v>
       </c>
     </row>
-    <row r="84" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="84" spans="2:7">
       <c r="B84" s="1">
         <v>46798</v>
       </c>
@@ -2160,7 +2142,7 @@
         <v>4.3029999999999999</v>
       </c>
     </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="85" spans="2:7">
       <c r="B85" s="1">
         <v>46798</v>
       </c>
@@ -2180,7 +2162,7 @@
         <v>4.3049999999999997</v>
       </c>
     </row>
-    <row r="86" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="86" spans="2:7">
       <c r="B86" s="1">
         <v>46812</v>
       </c>
@@ -2200,7 +2182,7 @@
         <v>4.306</v>
       </c>
     </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="87" spans="2:7">
       <c r="B87" s="1">
         <v>46812</v>
       </c>
@@ -2220,7 +2202,7 @@
         <v>4.2949999999999999</v>
       </c>
     </row>
-    <row r="88" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="88" spans="2:7">
       <c r="B88" s="1">
         <v>46812</v>
       </c>
@@ -2240,7 +2222,7 @@
         <v>4.319</v>
       </c>
     </row>
-    <row r="89" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="89" spans="2:7">
       <c r="B89" s="1">
         <v>46827</v>
       </c>
@@ -2260,7 +2242,7 @@
         <v>4.3150000000000004</v>
       </c>
     </row>
-    <row r="90" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="90" spans="2:7">
       <c r="B90" s="1">
         <v>46843</v>
       </c>
@@ -2280,7 +2262,7 @@
         <v>4.3319999999999999</v>
       </c>
     </row>
-    <row r="91" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="91" spans="2:7">
       <c r="B91" s="1">
         <v>46843</v>
       </c>
@@ -2300,7 +2282,7 @@
         <v>4.33</v>
       </c>
     </row>
-    <row r="92" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="92" spans="2:7">
       <c r="B92" s="1">
         <v>46843</v>
       </c>
@@ -2320,7 +2302,7 @@
         <v>4.3289999999999997</v>
       </c>
     </row>
-    <row r="93" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="93" spans="2:7">
       <c r="B93" s="1">
         <v>46858</v>
       </c>
@@ -2340,7 +2322,7 @@
         <v>4.335</v>
       </c>
     </row>
-    <row r="94" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="94" spans="2:7">
       <c r="B94" s="1">
         <v>46873</v>
       </c>
@@ -2360,7 +2342,7 @@
         <v>4.3540000000000001</v>
       </c>
     </row>
-    <row r="95" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="95" spans="2:7">
       <c r="B95" s="1">
         <v>46873</v>
       </c>
@@ -2380,7 +2362,7 @@
         <v>4.343</v>
       </c>
     </row>
-    <row r="96" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="96" spans="2:7">
       <c r="B96" s="1">
         <v>46873</v>
       </c>
@@ -2400,7 +2382,7 @@
         <v>4.3470000000000004</v>
       </c>
     </row>
-    <row r="97" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="97" spans="2:7">
       <c r="B97" s="1">
         <v>46888</v>
       </c>
@@ -2420,7 +2402,7 @@
         <v>4.3499999999999996</v>
       </c>
     </row>
-    <row r="98" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="98" spans="2:7">
       <c r="B98" s="1">
         <v>46888</v>
       </c>
@@ -2440,7 +2422,7 @@
         <v>4.335</v>
       </c>
     </row>
-    <row r="99" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="99" spans="2:7">
       <c r="B99" s="1">
         <v>46904</v>
       </c>
@@ -2460,7 +2442,7 @@
         <v>4.3570000000000002</v>
       </c>
     </row>
-    <row r="100" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="100" spans="2:7">
       <c r="B100" s="1">
         <v>46904</v>
       </c>
@@ -2480,7 +2462,7 @@
         <v>4.3479999999999999</v>
       </c>
     </row>
-    <row r="101" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="101" spans="2:7">
       <c r="B101" s="1">
         <v>46904</v>
       </c>
@@ -2500,7 +2482,7 @@
         <v>4.343</v>
       </c>
     </row>
-    <row r="102" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="102" spans="2:7">
       <c r="B102" s="1">
         <v>46919</v>
       </c>
@@ -2520,7 +2502,7 @@
         <v>4.3540000000000001</v>
       </c>
     </row>
-    <row r="103" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="103" spans="2:7">
       <c r="B103" s="1">
         <v>46934</v>
       </c>
@@ -2540,7 +2522,7 @@
         <v>4.3659999999999997</v>
       </c>
     </row>
-    <row r="104" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="104" spans="2:7">
       <c r="B104" s="1">
         <v>46934</v>
       </c>
@@ -2560,7 +2542,7 @@
         <v>4.3600000000000003</v>
       </c>
     </row>
-    <row r="105" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="105" spans="2:7">
       <c r="B105" s="1">
         <v>46934</v>
       </c>
@@ -2580,7 +2562,7 @@
         <v>4.3620000000000001</v>
       </c>
     </row>
-    <row r="106" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="106" spans="2:7">
       <c r="B106" s="1">
         <v>46949</v>
       </c>
@@ -2600,7 +2582,7 @@
         <v>4.37</v>
       </c>
     </row>
-    <row r="107" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="107" spans="2:7">
       <c r="B107" s="1">
         <v>46965</v>
       </c>
@@ -2620,7 +2602,7 @@
         <v>4.3739999999999997</v>
       </c>
     </row>
-    <row r="108" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="108" spans="2:7">
       <c r="B108" s="1">
         <v>46965</v>
       </c>
@@ -2640,7 +2622,7 @@
         <v>4.3620000000000001</v>
       </c>
     </row>
-    <row r="109" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="109" spans="2:7">
       <c r="B109" s="1">
         <v>46965</v>
       </c>
@@ -2660,7 +2642,7 @@
         <v>4.3650000000000002</v>
       </c>
     </row>
-    <row r="110" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="110" spans="2:7">
       <c r="B110" s="1">
         <v>46980</v>
       </c>
@@ -2680,7 +2662,7 @@
         <v>4.3630000000000004</v>
       </c>
     </row>
-    <row r="111" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="111" spans="2:7">
       <c r="B111" s="1">
         <v>46980</v>
       </c>
@@ -2700,7 +2682,7 @@
         <v>4.3730000000000002</v>
       </c>
     </row>
-    <row r="112" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="112" spans="2:7">
       <c r="B112" s="1">
         <v>46980</v>
       </c>
@@ -2720,7 +2702,7 @@
         <v>4.3959999999999999</v>
       </c>
     </row>
-    <row r="113" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="113" spans="2:8">
       <c r="B113" s="1">
         <v>46996</v>
       </c>
@@ -2740,7 +2722,7 @@
         <v>4.3789999999999996</v>
       </c>
     </row>
-    <row r="114" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="114" spans="2:8">
       <c r="B114" s="1">
         <v>46996</v>
       </c>
@@ -2760,7 +2742,7 @@
         <v>4.3680000000000003</v>
       </c>
     </row>
-    <row r="115" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="115" spans="2:8">
       <c r="B115" s="1">
         <v>46996</v>
       </c>
@@ -2780,7 +2762,7 @@
         <v>4.37</v>
       </c>
     </row>
-    <row r="116" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="116" spans="2:8">
       <c r="B116" s="1">
         <v>47011</v>
       </c>
@@ -2800,7 +2782,7 @@
         <v>4.38</v>
       </c>
     </row>
-    <row r="117" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="117" spans="2:8">
       <c r="B117" s="1">
         <v>47026</v>
       </c>
@@ -2820,7 +2802,7 @@
         <v>4.3789999999999996</v>
       </c>
     </row>
-    <row r="118" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="118" spans="2:8">
       <c r="B118" s="1">
         <v>47026</v>
       </c>
@@ -2840,7 +2822,7 @@
         <v>4.3869999999999996</v>
       </c>
     </row>
-    <row r="119" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="119" spans="2:8">
       <c r="B119" s="1">
         <v>47041</v>
       </c>
@@ -2860,7 +2842,7 @@
         <v>4.391</v>
       </c>
     </row>
-    <row r="120" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="120" spans="2:8">
       <c r="B120" s="1">
         <v>47057</v>
       </c>
@@ -2880,7 +2862,7 @@
         <v>4.3869999999999996</v>
       </c>
     </row>
-    <row r="121" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="121" spans="2:8">
       <c r="B121" s="1">
         <v>47057</v>
       </c>
@@ -2900,7 +2882,7 @@
         <v>4.3860000000000001</v>
       </c>
     </row>
-    <row r="122" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="122" spans="2:8">
       <c r="B122" s="1">
         <v>47072</v>
       </c>
@@ -2920,7 +2902,7 @@
         <v>4.3920000000000003</v>
       </c>
     </row>
-    <row r="123" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="123" spans="2:8">
       <c r="B123" s="1">
         <v>47072</v>
       </c>
@@ -2940,7 +2922,7 @@
         <v>4.3920000000000003</v>
       </c>
     </row>
-    <row r="124" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="124" spans="2:8">
       <c r="B124" s="1">
         <v>47072</v>
       </c>
@@ -2960,7 +2942,7 @@
         <v>4.3940000000000001</v>
       </c>
     </row>
-    <row r="125" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="125" spans="2:8">
       <c r="B125" s="1">
         <v>47087</v>
       </c>
@@ -2980,7 +2962,7 @@
         <v>4.3979999999999997</v>
       </c>
     </row>
-    <row r="126" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="126" spans="2:8">
       <c r="B126" s="1">
         <v>47087</v>
       </c>
@@ -2999,8 +2981,9 @@
       <c r="G126" s="2">
         <v>4.3979999999999997</v>
       </c>
-    </row>
-    <row r="127" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="H126" s="13"/>
+    </row>
+    <row r="127" spans="2:8">
       <c r="B127" s="1">
         <v>47102</v>
       </c>
@@ -3020,7 +3003,7 @@
         <v>4.3970000000000002</v>
       </c>
     </row>
-    <row r="128" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="128" spans="2:8">
       <c r="B128" s="1">
         <v>47118</v>
       </c>
@@ -3040,7 +3023,7 @@
         <v>4.4039999999999999</v>
       </c>
     </row>
-    <row r="129" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="129" spans="2:7">
       <c r="B129" s="1">
         <v>47118</v>
       </c>
@@ -3060,7 +3043,7 @@
         <v>4.4020000000000001</v>
       </c>
     </row>
-    <row r="130" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="130" spans="2:7">
       <c r="B130" s="1">
         <v>47133</v>
       </c>
@@ -3080,7 +3063,7 @@
         <v>4.4139999999999997</v>
       </c>
     </row>
-    <row r="131" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="131" spans="2:7">
       <c r="B131" s="1">
         <v>47149</v>
       </c>
@@ -3100,7 +3083,7 @@
         <v>4.4139999999999997</v>
       </c>
     </row>
-    <row r="132" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="132" spans="2:7">
       <c r="B132" s="1">
         <v>47149</v>
       </c>
@@ -3120,7 +3103,7 @@
         <v>4.4119999999999999</v>
       </c>
     </row>
-    <row r="133" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="133" spans="2:7">
       <c r="B133" s="1">
         <v>47164</v>
       </c>
@@ -3140,7 +3123,7 @@
         <v>4.4160000000000004</v>
       </c>
     </row>
-    <row r="134" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="134" spans="2:7">
       <c r="B134" s="1">
         <v>47164</v>
       </c>
@@ -3160,7 +3143,7 @@
         <v>4.4189999999999996</v>
       </c>
     </row>
-    <row r="135" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="135" spans="2:7">
       <c r="B135" s="1">
         <v>47164</v>
       </c>
@@ -3180,7 +3163,7 @@
         <v>4.3129999999999997</v>
       </c>
     </row>
-    <row r="136" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="136" spans="2:7">
       <c r="B136" s="1">
         <v>47177</v>
       </c>
@@ -3200,7 +3183,7 @@
         <v>4.41</v>
       </c>
     </row>
-    <row r="137" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="137" spans="2:7">
       <c r="B137" s="1">
         <v>47177</v>
       </c>
@@ -3220,7 +3203,7 @@
         <v>4.4080000000000004</v>
       </c>
     </row>
-    <row r="138" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="138" spans="2:7">
       <c r="B138" s="1">
         <v>47192</v>
       </c>
@@ -3240,7 +3223,7 @@
         <v>4.407</v>
       </c>
     </row>
-    <row r="139" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="139" spans="2:7">
       <c r="B139" s="1">
         <v>47208</v>
       </c>
@@ -3260,7 +3243,7 @@
         <v>4.4260000000000002</v>
       </c>
     </row>
-    <row r="140" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="140" spans="2:7">
       <c r="B140" s="1">
         <v>47208</v>
       </c>
@@ -3280,7 +3263,7 @@
         <v>4.4169999999999998</v>
       </c>
     </row>
-    <row r="141" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="141" spans="2:7">
       <c r="B141" s="1">
         <v>47223</v>
       </c>
@@ -3300,7 +3283,7 @@
         <v>4.4260000000000002</v>
       </c>
     </row>
-    <row r="142" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="142" spans="2:7">
       <c r="B142" s="1">
         <v>47238</v>
       </c>
@@ -3320,7 +3303,7 @@
         <v>4.4269999999999996</v>
       </c>
     </row>
-    <row r="143" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="143" spans="2:7">
       <c r="B143" s="1">
         <v>47238</v>
       </c>
@@ -3340,7 +3323,7 @@
         <v>4.42</v>
       </c>
     </row>
-    <row r="144" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="144" spans="2:7">
       <c r="B144" s="1">
         <v>47253</v>
       </c>
@@ -3360,7 +3343,7 @@
         <v>4.4219999999999997</v>
       </c>
     </row>
-    <row r="145" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="145" spans="2:7">
       <c r="B145" s="1">
         <v>47253</v>
       </c>
@@ -3380,7 +3363,7 @@
         <v>4.4269999999999996</v>
       </c>
     </row>
-    <row r="146" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="146" spans="2:7">
       <c r="B146" s="1">
         <v>47269</v>
       </c>
@@ -3400,7 +3383,7 @@
         <v>4.4329999999999998</v>
       </c>
     </row>
-    <row r="147" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="147" spans="2:7">
       <c r="B147" s="1">
         <v>47269</v>
       </c>
@@ -3420,7 +3403,7 @@
         <v>4.43</v>
       </c>
     </row>
-    <row r="148" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="148" spans="2:7">
       <c r="B148" s="1">
         <v>47284</v>
       </c>
@@ -3440,7 +3423,7 @@
         <v>4.4320000000000004</v>
       </c>
     </row>
-    <row r="149" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="149" spans="2:7">
       <c r="B149" s="1">
         <v>47299</v>
       </c>
@@ -3460,7 +3443,7 @@
         <v>4.444</v>
       </c>
     </row>
-    <row r="150" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="150" spans="2:7">
       <c r="B150" s="1">
         <v>47299</v>
       </c>
@@ -3480,7 +3463,7 @@
         <v>4.4359999999999999</v>
       </c>
     </row>
-    <row r="151" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="151" spans="2:7">
       <c r="B151" s="1">
         <v>47314</v>
       </c>
@@ -3500,7 +3483,7 @@
         <v>4.4420000000000002</v>
       </c>
     </row>
-    <row r="152" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="152" spans="2:7">
       <c r="B152" s="1">
         <v>47330</v>
       </c>
@@ -3520,7 +3503,7 @@
         <v>4.444</v>
       </c>
     </row>
-    <row r="153" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="153" spans="2:7">
       <c r="B153" s="1">
         <v>47330</v>
       </c>
@@ -3540,7 +3523,7 @@
         <v>4.4459999999999997</v>
       </c>
     </row>
-    <row r="154" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="154" spans="2:7">
       <c r="B154" s="1">
         <v>47345</v>
       </c>
@@ -3560,7 +3543,7 @@
         <v>4.43</v>
       </c>
     </row>
-    <row r="155" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="155" spans="2:7">
       <c r="B155" s="1">
         <v>47345</v>
       </c>
@@ -3580,7 +3563,7 @@
         <v>4.444</v>
       </c>
     </row>
-    <row r="156" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="156" spans="2:7">
       <c r="B156" s="1">
         <v>47345</v>
       </c>
@@ -3600,7 +3583,7 @@
         <v>4.4480000000000004</v>
       </c>
     </row>
-    <row r="157" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="157" spans="2:7">
       <c r="B157" s="1">
         <v>47361</v>
       </c>
@@ -3620,7 +3603,7 @@
         <v>4.4459999999999997</v>
       </c>
     </row>
-    <row r="158" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="158" spans="2:7">
       <c r="B158" s="1">
         <v>47361</v>
       </c>
@@ -3640,7 +3623,7 @@
         <v>4.4509999999999996</v>
       </c>
     </row>
-    <row r="159" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="159" spans="2:7">
       <c r="B159" s="1">
         <v>47391</v>
       </c>
@@ -3660,7 +3643,7 @@
         <v>4.4569999999999999</v>
       </c>
     </row>
-    <row r="160" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="160" spans="2:7">
       <c r="B160" s="1">
         <v>47391</v>
       </c>
@@ -3680,7 +3663,7 @@
         <v>4.4539999999999997</v>
       </c>
     </row>
-    <row r="161" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="161" spans="2:7">
       <c r="B161" s="1">
         <v>47422</v>
       </c>
@@ -3700,7 +3683,7 @@
         <v>4.4640000000000004</v>
       </c>
     </row>
-    <row r="162" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="162" spans="2:7">
       <c r="B162" s="1">
         <v>47422</v>
       </c>
@@ -3720,7 +3703,7 @@
         <v>4.4619999999999997</v>
       </c>
     </row>
-    <row r="163" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="163" spans="2:7">
       <c r="B163" s="1">
         <v>47437</v>
       </c>
@@ -3740,7 +3723,7 @@
         <v>4.4550000000000001</v>
       </c>
     </row>
-    <row r="164" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="164" spans="2:7">
       <c r="B164" s="1">
         <v>47452</v>
       </c>
@@ -3760,7 +3743,7 @@
         <v>4.4640000000000004</v>
       </c>
     </row>
-    <row r="165" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="165" spans="2:7">
       <c r="B165" s="1">
         <v>47452</v>
       </c>
@@ -3780,7 +3763,7 @@
         <v>4.4669999999999996</v>
       </c>
     </row>
-    <row r="166" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="166" spans="2:7">
       <c r="B166" s="1">
         <v>47483</v>
       </c>
@@ -3800,7 +3783,7 @@
         <v>4.476</v>
       </c>
     </row>
-    <row r="167" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="167" spans="2:7">
       <c r="B167" s="1">
         <v>47483</v>
       </c>
@@ -3820,7 +3803,7 @@
         <v>4.4729999999999999</v>
       </c>
     </row>
-    <row r="168" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="168" spans="2:7">
       <c r="B168" s="1">
         <v>47514</v>
       </c>
@@ -3840,7 +3823,7 @@
         <v>4.4870000000000001</v>
       </c>
     </row>
-    <row r="169" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="169" spans="2:7">
       <c r="B169" s="1">
         <v>47514</v>
       </c>
@@ -3860,7 +3843,7 @@
         <v>4.4790000000000001</v>
       </c>
     </row>
-    <row r="170" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="170" spans="2:7">
       <c r="B170" s="1">
         <v>47529</v>
       </c>
@@ -3880,7 +3863,7 @@
         <v>4.4720000000000004</v>
       </c>
     </row>
-    <row r="171" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="171" spans="2:7">
       <c r="B171" s="1">
         <v>47542</v>
       </c>
@@ -3900,7 +3883,7 @@
         <v>4.4749999999999996</v>
       </c>
     </row>
-    <row r="172" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="172" spans="2:7">
       <c r="B172" s="1">
         <v>47573</v>
       </c>
@@ -3920,7 +3903,7 @@
         <v>4.4859999999999998</v>
       </c>
     </row>
-    <row r="173" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="173" spans="2:7">
       <c r="B173" s="1">
         <v>47573</v>
       </c>
@@ -3940,7 +3923,7 @@
         <v>4.4859999999999998</v>
       </c>
     </row>
-    <row r="174" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="174" spans="2:7">
       <c r="B174" s="1">
         <v>47603</v>
       </c>
@@ -3960,7 +3943,7 @@
         <v>4.492</v>
       </c>
     </row>
-    <row r="175" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="175" spans="2:7">
       <c r="B175" s="1">
         <v>47603</v>
       </c>
@@ -3980,7 +3963,7 @@
         <v>4.484</v>
       </c>
     </row>
-    <row r="176" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="176" spans="2:7">
       <c r="B176" s="1">
         <v>47618</v>
       </c>
@@ -4000,7 +3983,7 @@
         <v>4.492</v>
       </c>
     </row>
-    <row r="177" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="177" spans="2:7">
       <c r="B177" s="1">
         <v>47618</v>
       </c>
@@ -4020,7 +4003,7 @@
         <v>4.4880000000000004</v>
       </c>
     </row>
-    <row r="178" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="178" spans="2:7">
       <c r="B178" s="1">
         <v>47634</v>
       </c>
@@ -4040,7 +4023,7 @@
         <v>4.5010000000000003</v>
       </c>
     </row>
-    <row r="179" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="179" spans="2:7">
       <c r="B179" s="1">
         <v>47634</v>
       </c>
@@ -4060,7 +4043,7 @@
         <v>4.4980000000000002</v>
       </c>
     </row>
-    <row r="180" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="180" spans="2:7">
       <c r="B180" s="1">
         <v>47664</v>
       </c>
@@ -4080,7 +4063,7 @@
         <v>4.5039999999999996</v>
       </c>
     </row>
-    <row r="181" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="181" spans="2:7">
       <c r="B181" s="1">
         <v>47664</v>
       </c>
@@ -4100,7 +4083,7 @@
         <v>4.4960000000000004</v>
       </c>
     </row>
-    <row r="182" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="182" spans="2:7">
       <c r="B182" s="1">
         <v>47695</v>
       </c>
@@ -4120,7 +4103,7 @@
         <v>4.5039999999999996</v>
       </c>
     </row>
-    <row r="183" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="183" spans="2:7">
       <c r="B183" s="1">
         <v>47695</v>
       </c>
@@ -4140,7 +4123,7 @@
         <v>4.5030000000000001</v>
       </c>
     </row>
-    <row r="184" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="184" spans="2:7">
       <c r="B184" s="1">
         <v>47710</v>
       </c>
@@ -4160,7 +4143,7 @@
         <v>4.5030000000000001</v>
       </c>
     </row>
-    <row r="185" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="185" spans="2:7">
       <c r="B185" s="1">
         <v>47726</v>
       </c>
@@ -4180,7 +4163,7 @@
         <v>4.5110000000000001</v>
       </c>
     </row>
-    <row r="186" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="186" spans="2:7">
       <c r="B186" s="1">
         <v>47726</v>
       </c>
@@ -4200,7 +4183,7 @@
         <v>4.5060000000000002</v>
       </c>
     </row>
-    <row r="187" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="187" spans="2:7">
       <c r="B187" s="1">
         <v>47756</v>
       </c>
@@ -4220,7 +4203,7 @@
         <v>4.5090000000000003</v>
       </c>
     </row>
-    <row r="188" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="188" spans="2:7">
       <c r="B188" s="1">
         <v>47756</v>
       </c>
@@ -4240,7 +4223,7 @@
         <v>4.5090000000000003</v>
       </c>
     </row>
-    <row r="189" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="189" spans="2:7">
       <c r="B189" s="1">
         <v>47787</v>
       </c>
@@ -4260,7 +4243,7 @@
         <v>4.5179999999999998</v>
       </c>
     </row>
-    <row r="190" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="190" spans="2:7">
       <c r="B190" s="1">
         <v>47787</v>
       </c>
@@ -4280,7 +4263,7 @@
         <v>4.5119999999999996</v>
       </c>
     </row>
-    <row r="191" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="191" spans="2:7">
       <c r="B191" s="1">
         <v>47802</v>
       </c>
@@ -4300,7 +4283,7 @@
         <v>4.5179999999999998</v>
       </c>
     </row>
-    <row r="192" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="192" spans="2:7">
       <c r="B192" s="1">
         <v>47817</v>
       </c>
@@ -4320,7 +4303,7 @@
         <v>4.524</v>
       </c>
     </row>
-    <row r="193" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="193" spans="2:7">
       <c r="B193" s="1">
         <v>47817</v>
       </c>
@@ -4340,7 +4323,7 @@
         <v>4.5209999999999999</v>
       </c>
     </row>
-    <row r="194" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="194" spans="2:7">
       <c r="B194" s="1">
         <v>47848</v>
       </c>
@@ -4360,7 +4343,7 @@
         <v>4.5250000000000004</v>
       </c>
     </row>
-    <row r="195" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="195" spans="2:7">
       <c r="B195" s="1">
         <v>47848</v>
       </c>
@@ -4380,7 +4363,7 @@
         <v>4.5270000000000001</v>
       </c>
     </row>
-    <row r="196" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="196" spans="2:7">
       <c r="B196" s="1">
         <v>47879</v>
       </c>
@@ -4400,7 +4383,7 @@
         <v>4.5279999999999996</v>
       </c>
     </row>
-    <row r="197" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="197" spans="2:7">
       <c r="B197" s="1">
         <v>47879</v>
       </c>
@@ -4420,7 +4403,7 @@
         <v>4.5279999999999996</v>
       </c>
     </row>
-    <row r="198" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="198" spans="2:7">
       <c r="B198" s="1">
         <v>47894</v>
       </c>
@@ -4440,7 +4423,7 @@
         <v>4.5010000000000003</v>
       </c>
     </row>
-    <row r="199" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="199" spans="2:7">
       <c r="B199" s="1">
         <v>47894</v>
       </c>
@@ -4460,7 +4443,7 @@
         <v>4.51</v>
       </c>
     </row>
-    <row r="200" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="200" spans="2:7">
       <c r="B200" s="1">
         <v>47907</v>
       </c>
@@ -4480,7 +4463,7 @@
         <v>4.524</v>
       </c>
     </row>
-    <row r="201" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="201" spans="2:7">
       <c r="B201" s="1">
         <v>47907</v>
       </c>
@@ -4500,7 +4483,7 @@
         <v>4.53</v>
       </c>
     </row>
-    <row r="202" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="202" spans="2:7">
       <c r="B202" s="1">
         <v>47938</v>
       </c>
@@ -4520,7 +4503,7 @@
         <v>4.5279999999999996</v>
       </c>
     </row>
-    <row r="203" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="203" spans="2:7">
       <c r="B203" s="1">
         <v>47938</v>
       </c>
@@ -4540,7 +4523,7 @@
         <v>4.5339999999999998</v>
       </c>
     </row>
-    <row r="204" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="204" spans="2:7">
       <c r="B204" s="1">
         <v>47968</v>
       </c>
@@ -4560,7 +4543,7 @@
         <v>4.5279999999999996</v>
       </c>
     </row>
-    <row r="205" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="205" spans="2:7">
       <c r="B205" s="1">
         <v>47968</v>
       </c>
@@ -4580,7 +4563,7 @@
         <v>4.5350000000000001</v>
       </c>
     </row>
-    <row r="206" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="206" spans="2:7">
       <c r="B206" s="1">
         <v>47983</v>
       </c>
@@ -4600,7 +4583,7 @@
         <v>4.5380000000000003</v>
       </c>
     </row>
-    <row r="207" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="207" spans="2:7">
       <c r="B207" s="1">
         <v>47999</v>
       </c>
@@ -4620,7 +4603,7 @@
         <v>4.5369999999999999</v>
       </c>
     </row>
-    <row r="208" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="208" spans="2:7">
       <c r="B208" s="1">
         <v>47999</v>
       </c>
@@ -4640,7 +4623,7 @@
         <v>4.5439999999999996</v>
       </c>
     </row>
-    <row r="209" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="209" spans="2:7">
       <c r="B209" s="1">
         <v>48029</v>
       </c>
@@ -4660,7 +4643,7 @@
         <v>4.5359999999999996</v>
       </c>
     </row>
-    <row r="210" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="210" spans="2:7">
       <c r="B210" s="1">
         <v>48029</v>
       </c>
@@ -4680,7 +4663,7 @@
         <v>4.5460000000000003</v>
       </c>
     </row>
-    <row r="211" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="211" spans="2:7">
       <c r="B211" s="1">
         <v>48060</v>
       </c>
@@ -4700,7 +4683,7 @@
         <v>4.55</v>
       </c>
     </row>
-    <row r="212" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="212" spans="2:7">
       <c r="B212" s="1">
         <v>48060</v>
       </c>
@@ -4720,7 +4703,7 @@
         <v>4.5419999999999998</v>
       </c>
     </row>
-    <row r="213" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="213" spans="2:7">
       <c r="B213" s="1">
         <v>48075</v>
       </c>
@@ -4740,7 +4723,7 @@
         <v>4.5570000000000004</v>
       </c>
     </row>
-    <row r="214" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="214" spans="2:7">
       <c r="B214" s="1">
         <v>48091</v>
       </c>
@@ -4760,7 +4743,7 @@
         <v>4.556</v>
       </c>
     </row>
-    <row r="215" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="215" spans="2:7">
       <c r="B215" s="1">
         <v>48091</v>
       </c>
@@ -4780,7 +4763,7 @@
         <v>4.5410000000000004</v>
       </c>
     </row>
-    <row r="216" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="216" spans="2:7">
       <c r="B216" s="1">
         <v>48121</v>
       </c>
@@ -4800,7 +4783,7 @@
         <v>4.5529999999999999</v>
       </c>
     </row>
-    <row r="217" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="217" spans="2:7">
       <c r="B217" s="1">
         <v>48152</v>
       </c>
@@ -4820,7 +4803,7 @@
         <v>4.5590000000000002</v>
       </c>
     </row>
-    <row r="218" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="218" spans="2:7">
       <c r="B218" s="1">
         <v>48167</v>
       </c>
@@ -4840,7 +4823,7 @@
         <v>4.5750000000000002</v>
       </c>
     </row>
-    <row r="219" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="219" spans="2:7">
       <c r="B219" s="1">
         <v>48182</v>
       </c>
@@ -4860,7 +4843,7 @@
         <v>4.5650000000000004</v>
       </c>
     </row>
-    <row r="220" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="220" spans="2:7">
       <c r="B220" s="1">
         <v>48213</v>
       </c>
@@ -4880,7 +4863,7 @@
         <v>4.5670000000000002</v>
       </c>
     </row>
-    <row r="221" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="221" spans="2:7">
       <c r="B221" s="1">
         <v>48244</v>
       </c>
@@ -4900,7 +4883,7 @@
         <v>4.5759999999999996</v>
       </c>
     </row>
-    <row r="222" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="222" spans="2:7">
       <c r="B222" s="1">
         <v>48259</v>
       </c>
@@ -4920,7 +4903,7 @@
         <v>4.59</v>
       </c>
     </row>
-    <row r="223" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="223" spans="2:7">
       <c r="B223" s="1">
         <v>48273</v>
       </c>
@@ -4940,7 +4923,7 @@
         <v>4.5759999999999996</v>
       </c>
     </row>
-    <row r="224" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="224" spans="2:7">
       <c r="B224" s="1">
         <v>48304</v>
       </c>
@@ -4960,7 +4943,7 @@
         <v>4.5810000000000004</v>
       </c>
     </row>
-    <row r="225" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="225" spans="2:7">
       <c r="B225" s="1">
         <v>48334</v>
       </c>
@@ -4980,7 +4963,7 @@
         <v>4.585</v>
       </c>
     </row>
-    <row r="226" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="226" spans="2:7">
       <c r="B226" s="1">
         <v>48349</v>
       </c>
@@ -5000,7 +4983,7 @@
         <v>4.5970000000000004</v>
       </c>
     </row>
-    <row r="227" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="227" spans="2:7">
       <c r="B227" s="1">
         <v>48365</v>
       </c>
@@ -5020,7 +5003,7 @@
         <v>4.5910000000000002</v>
       </c>
     </row>
-    <row r="228" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="228" spans="2:7">
       <c r="B228" s="1">
         <v>48395</v>
       </c>
@@ -5040,7 +5023,7 @@
         <v>4.5919999999999996</v>
       </c>
     </row>
-    <row r="229" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="229" spans="2:7">
       <c r="B229" s="1">
         <v>48426</v>
       </c>
@@ -5060,7 +5043,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="230" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="230" spans="2:7">
       <c r="B230" s="1">
         <v>48441</v>
       </c>
@@ -5080,7 +5063,7 @@
         <v>4.6029999999999998</v>
       </c>
     </row>
-    <row r="231" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="231" spans="2:7">
       <c r="B231" s="1">
         <v>48457</v>
       </c>
@@ -5100,7 +5083,7 @@
         <v>4.601</v>
       </c>
     </row>
-    <row r="232" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="232" spans="2:7">
       <c r="B232" s="1">
         <v>48487</v>
       </c>
@@ -5120,7 +5103,7 @@
         <v>4.6100000000000003</v>
       </c>
     </row>
-    <row r="233" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="233" spans="2:7">
       <c r="B233" s="1">
         <v>48518</v>
       </c>
@@ -5140,7 +5123,7 @@
         <v>4.6150000000000002</v>
       </c>
     </row>
-    <row r="234" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="234" spans="2:7">
       <c r="B234" s="1">
         <v>48533</v>
       </c>
@@ -5160,7 +5143,7 @@
         <v>4.6139999999999999</v>
       </c>
     </row>
-    <row r="235" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="235" spans="2:7">
       <c r="B235" s="1">
         <v>48548</v>
       </c>
@@ -5180,7 +5163,7 @@
         <v>4.6189999999999998</v>
       </c>
     </row>
-    <row r="236" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="236" spans="2:7">
       <c r="B236" s="1">
         <v>48579</v>
       </c>
@@ -5200,7 +5183,7 @@
         <v>4.6210000000000004</v>
       </c>
     </row>
-    <row r="237" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="237" spans="2:7">
       <c r="B237" s="1">
         <v>48610</v>
       </c>
@@ -5220,7 +5203,7 @@
         <v>4.6260000000000003</v>
       </c>
     </row>
-    <row r="238" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="238" spans="2:7">
       <c r="B238" s="1">
         <v>48625</v>
       </c>
@@ -5240,7 +5223,7 @@
         <v>4.6340000000000003</v>
       </c>
     </row>
-    <row r="239" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="239" spans="2:7">
       <c r="B239" s="1">
         <v>48638</v>
       </c>
@@ -5260,7 +5243,7 @@
         <v>4.625</v>
       </c>
     </row>
-    <row r="240" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="240" spans="2:7">
       <c r="B240" s="1">
         <v>48669</v>
       </c>
@@ -5280,7 +5263,7 @@
         <v>4.63</v>
       </c>
     </row>
-    <row r="241" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="241" spans="2:7">
       <c r="B241" s="1">
         <v>48699</v>
       </c>
@@ -5300,7 +5283,7 @@
         <v>4.6390000000000002</v>
       </c>
     </row>
-    <row r="242" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="242" spans="2:7">
       <c r="B242" s="1">
         <v>48714</v>
       </c>
@@ -5320,7 +5303,7 @@
         <v>4.6440000000000001</v>
       </c>
     </row>
-    <row r="243" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="243" spans="2:7">
       <c r="B243" s="1">
         <v>48730</v>
       </c>
@@ -5340,7 +5323,7 @@
         <v>4.6420000000000003</v>
       </c>
     </row>
-    <row r="244" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="244" spans="2:7">
       <c r="B244" s="1">
         <v>48760</v>
       </c>
@@ -5360,7 +5343,7 @@
         <v>4.6440000000000001</v>
       </c>
     </row>
-    <row r="245" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="245" spans="2:7">
       <c r="B245" s="1">
         <v>48791</v>
       </c>
@@ -5380,7 +5363,7 @@
         <v>4.6500000000000004</v>
       </c>
     </row>
-    <row r="246" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="246" spans="2:7">
       <c r="B246" s="1">
         <v>48806</v>
       </c>
@@ -5400,7 +5383,7 @@
         <v>4.657</v>
       </c>
     </row>
-    <row r="247" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="247" spans="2:7">
       <c r="B247" s="1">
         <v>48822</v>
       </c>
@@ -5420,7 +5403,7 @@
         <v>4.6520000000000001</v>
       </c>
     </row>
-    <row r="248" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="248" spans="2:7">
       <c r="B248" s="1">
         <v>48898</v>
       </c>
@@ -5440,7 +5423,7 @@
         <v>4.6669999999999998</v>
       </c>
     </row>
-    <row r="249" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="249" spans="2:7">
       <c r="B249" s="1">
         <v>48990</v>
       </c>
@@ -5460,7 +5443,7 @@
         <v>4.6829999999999998</v>
       </c>
     </row>
-    <row r="250" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="250" spans="2:7">
       <c r="B250" s="1">
         <v>49079</v>
       </c>
@@ -5480,7 +5463,7 @@
         <v>4.6859999999999999</v>
       </c>
     </row>
-    <row r="251" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="251" spans="2:7">
       <c r="B251" s="1">
         <v>49171</v>
       </c>
@@ -5500,7 +5483,7 @@
         <v>4.7039999999999997</v>
       </c>
     </row>
-    <row r="252" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="252" spans="2:7">
       <c r="B252" s="1">
         <v>49263</v>
       </c>
@@ -5520,7 +5503,7 @@
         <v>4.7149999999999999</v>
       </c>
     </row>
-    <row r="253" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="253" spans="2:7">
       <c r="B253" s="1">
         <v>49355</v>
       </c>
@@ -5540,7 +5523,7 @@
         <v>4.7240000000000002</v>
       </c>
     </row>
-    <row r="254" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="254" spans="2:7">
       <c r="B254" s="1">
         <v>49444</v>
       </c>
@@ -5560,7 +5543,7 @@
         <v>4.734</v>
       </c>
     </row>
-    <row r="255" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="255" spans="2:7">
       <c r="B255" s="1">
         <v>49536</v>
       </c>
@@ -5580,7 +5563,7 @@
         <v>4.7480000000000002</v>
       </c>
     </row>
-    <row r="256" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="256" spans="2:7">
       <c r="B256" s="1">
         <v>49628</v>
       </c>
@@ -5600,7 +5583,7 @@
         <v>4.7549999999999999</v>
       </c>
     </row>
-    <row r="257" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="257" spans="2:7">
       <c r="B257" s="1">
         <v>49720</v>
       </c>
@@ -5620,7 +5603,7 @@
         <v>4.7629999999999999</v>
       </c>
     </row>
-    <row r="258" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="258" spans="2:7">
       <c r="B258" s="1">
         <v>49720</v>
       </c>
@@ -5640,7 +5623,7 @@
         <v>4.665</v>
       </c>
     </row>
-    <row r="259" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="259" spans="2:7">
       <c r="B259" s="1">
         <v>49810</v>
       </c>
@@ -5660,7 +5643,7 @@
         <v>4.7720000000000002</v>
       </c>
     </row>
-    <row r="260" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="260" spans="2:7">
       <c r="B260" s="1">
         <v>49902</v>
       </c>
@@ -5680,7 +5663,7 @@
         <v>4.7770000000000001</v>
       </c>
     </row>
-    <row r="261" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="261" spans="2:7">
       <c r="B261" s="1">
         <v>50086</v>
       </c>
@@ -5700,7 +5683,7 @@
         <v>4.7350000000000003</v>
       </c>
     </row>
-    <row r="262" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="262" spans="2:7">
       <c r="B262" s="1">
         <v>50175</v>
       </c>
@@ -5720,7 +5703,7 @@
         <v>4.7320000000000002</v>
       </c>
     </row>
-    <row r="263" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="263" spans="2:7">
       <c r="B263" s="1">
         <v>50451</v>
       </c>
@@ -5740,7 +5723,7 @@
         <v>4.7610000000000001</v>
       </c>
     </row>
-    <row r="264" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="264" spans="2:7">
       <c r="B264" s="1">
         <v>50540</v>
       </c>
@@ -5760,7 +5743,7 @@
         <v>4.798</v>
       </c>
     </row>
-    <row r="265" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="265" spans="2:7">
       <c r="B265" s="1">
         <v>50816</v>
       </c>
@@ -5780,7 +5763,7 @@
         <v>4.8579999999999997</v>
       </c>
     </row>
-    <row r="266" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="266" spans="2:7">
       <c r="B266" s="1">
         <v>50905</v>
       </c>
@@ -5800,7 +5783,7 @@
         <v>4.9020000000000001</v>
       </c>
     </row>
-    <row r="267" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="267" spans="2:7">
       <c r="B267" s="1">
         <v>50997</v>
       </c>
@@ -5820,7 +5803,7 @@
         <v>4.9329999999999998</v>
       </c>
     </row>
-    <row r="268" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="268" spans="2:7">
       <c r="B268" s="1">
         <v>51089</v>
       </c>
@@ -5840,7 +5823,7 @@
         <v>4.9569999999999999</v>
       </c>
     </row>
-    <row r="269" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="269" spans="2:7">
       <c r="B269" s="1">
         <v>51181</v>
       </c>
@@ -5860,7 +5843,7 @@
         <v>4.9649999999999999</v>
       </c>
     </row>
-    <row r="270" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="270" spans="2:7">
       <c r="B270" s="1">
         <v>51271</v>
       </c>
@@ -5880,7 +5863,7 @@
         <v>5.05</v>
       </c>
     </row>
-    <row r="271" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="271" spans="2:7">
       <c r="B271" s="1">
         <v>51271</v>
       </c>
@@ -5900,7 +5883,7 @@
         <v>4.9820000000000002</v>
       </c>
     </row>
-    <row r="272" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="272" spans="2:7">
       <c r="B272" s="1">
         <v>51363</v>
       </c>
@@ -5920,7 +5903,7 @@
         <v>5.069</v>
       </c>
     </row>
-    <row r="273" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="273" spans="2:7">
       <c r="B273" s="1">
         <v>51363</v>
       </c>
@@ -5940,7 +5923,7 @@
         <v>5.0049999999999999</v>
       </c>
     </row>
-    <row r="274" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="274" spans="2:7">
       <c r="B274" s="1">
         <v>51455</v>
       </c>
@@ -5960,7 +5943,7 @@
         <v>5.0860000000000003</v>
       </c>
     </row>
-    <row r="275" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="275" spans="2:7">
       <c r="B275" s="1">
         <v>51455</v>
       </c>
@@ -5980,7 +5963,7 @@
         <v>5.0190000000000001</v>
       </c>
     </row>
-    <row r="276" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="276" spans="2:7">
       <c r="B276" s="1">
         <v>51547</v>
       </c>
@@ -6000,7 +5983,7 @@
         <v>5.0910000000000002</v>
       </c>
     </row>
-    <row r="277" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="277" spans="2:7">
       <c r="B277" s="1">
         <v>51547</v>
       </c>
@@ -6020,7 +6003,7 @@
         <v>5.0369999999999999</v>
       </c>
     </row>
-    <row r="278" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="278" spans="2:7">
       <c r="B278" s="1">
         <v>51636</v>
       </c>
@@ -6040,7 +6023,7 @@
         <v>5.1050000000000004</v>
       </c>
     </row>
-    <row r="279" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="279" spans="2:7">
       <c r="B279" s="1">
         <v>51636</v>
       </c>
@@ -6060,7 +6043,7 @@
         <v>5.0549999999999997</v>
       </c>
     </row>
-    <row r="280" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="280" spans="2:7">
       <c r="B280" s="1">
         <v>51728</v>
       </c>
@@ -6080,7 +6063,7 @@
         <v>5.1319999999999997</v>
       </c>
     </row>
-    <row r="281" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="281" spans="2:7">
       <c r="B281" s="1">
         <v>51728</v>
       </c>
@@ -6100,7 +6083,7 @@
         <v>5.0810000000000004</v>
       </c>
     </row>
-    <row r="282" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="282" spans="2:7">
       <c r="B282" s="1">
         <v>51820</v>
       </c>
@@ -6120,7 +6103,7 @@
         <v>5.1100000000000003</v>
       </c>
     </row>
-    <row r="283" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="283" spans="2:7">
       <c r="B283" s="1">
         <v>51835</v>
       </c>
@@ -6140,7 +6123,7 @@
         <v>5.1470000000000002</v>
       </c>
     </row>
-    <row r="284" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="284" spans="2:7">
       <c r="B284" s="1">
         <v>51912</v>
       </c>
@@ -6160,7 +6143,7 @@
         <v>5.1539999999999999</v>
       </c>
     </row>
-    <row r="285" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="285" spans="2:7">
       <c r="B285" s="1">
         <v>51912</v>
       </c>
@@ -6180,7 +6163,7 @@
         <v>5.133</v>
       </c>
     </row>
-    <row r="286" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="286" spans="2:7">
       <c r="B286" s="1">
         <v>52001</v>
       </c>
@@ -6200,7 +6183,7 @@
         <v>5.1509999999999998</v>
       </c>
     </row>
-    <row r="287" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="287" spans="2:7">
       <c r="B287" s="1">
         <v>52001</v>
       </c>
@@ -6220,7 +6203,7 @@
         <v>5.15</v>
       </c>
     </row>
-    <row r="288" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="288" spans="2:7">
       <c r="B288" s="1">
         <v>52093</v>
       </c>
@@ -6240,7 +6223,7 @@
         <v>5.173</v>
       </c>
     </row>
-    <row r="289" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="289" spans="2:7">
       <c r="B289" s="1">
         <v>52093</v>
       </c>
@@ -6260,7 +6243,7 @@
         <v>5.16</v>
       </c>
     </row>
-    <row r="290" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="290" spans="2:7">
       <c r="B290" s="1">
         <v>52185</v>
       </c>
@@ -6280,7 +6263,7 @@
         <v>5.1879999999999997</v>
       </c>
     </row>
-    <row r="291" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="291" spans="2:7">
       <c r="B291" s="1">
         <v>52185</v>
       </c>
@@ -6300,7 +6283,7 @@
         <v>5.1680000000000001</v>
       </c>
     </row>
-    <row r="292" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="292" spans="2:7">
       <c r="B292" s="1">
         <v>52277</v>
       </c>
@@ -6320,7 +6303,7 @@
         <v>5.1950000000000003</v>
       </c>
     </row>
-    <row r="293" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="293" spans="2:7">
       <c r="B293" s="1">
         <v>52277</v>
       </c>
@@ -6340,7 +6323,7 @@
         <v>5.18</v>
       </c>
     </row>
-    <row r="294" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="294" spans="2:7">
       <c r="B294" s="1">
         <v>52366</v>
       </c>
@@ -6360,7 +6343,7 @@
         <v>5.2080000000000002</v>
       </c>
     </row>
-    <row r="295" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="295" spans="2:7">
       <c r="B295" s="1">
         <v>52366</v>
       </c>
@@ -6380,7 +6363,7 @@
         <v>5.19</v>
       </c>
     </row>
-    <row r="296" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="296" spans="2:7">
       <c r="B296" s="1">
         <v>52458</v>
       </c>
@@ -6400,7 +6383,7 @@
         <v>5.2110000000000003</v>
       </c>
     </row>
-    <row r="297" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="297" spans="2:7">
       <c r="B297" s="1">
         <v>52458</v>
       </c>
@@ -6420,7 +6403,7 @@
         <v>5.194</v>
       </c>
     </row>
-    <row r="298" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="298" spans="2:7">
       <c r="B298" s="1">
         <v>52550</v>
       </c>
@@ -6440,7 +6423,7 @@
         <v>5.2130000000000001</v>
       </c>
     </row>
-    <row r="299" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="299" spans="2:7">
       <c r="B299" s="1">
         <v>52550</v>
       </c>
@@ -6460,7 +6443,7 @@
         <v>5.1929999999999996</v>
       </c>
     </row>
-    <row r="300" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="300" spans="2:7">
       <c r="B300" s="1">
         <v>52642</v>
       </c>
@@ -6480,7 +6463,7 @@
         <v>5.226</v>
       </c>
     </row>
-    <row r="301" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="301" spans="2:7">
       <c r="B301" s="1">
         <v>52642</v>
       </c>
@@ -6500,7 +6483,7 @@
         <v>5.2110000000000003</v>
       </c>
     </row>
-    <row r="302" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="302" spans="2:7">
       <c r="B302" s="1">
         <v>52732</v>
       </c>
@@ -6520,7 +6503,7 @@
         <v>5.2370000000000001</v>
       </c>
     </row>
-    <row r="303" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="303" spans="2:7">
       <c r="B303" s="1">
         <v>52732</v>
       </c>
@@ -6540,7 +6523,7 @@
         <v>5.2130000000000001</v>
       </c>
     </row>
-    <row r="304" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="304" spans="2:7">
       <c r="B304" s="1">
         <v>52824</v>
       </c>
@@ -6560,7 +6543,7 @@
         <v>5.2530000000000001</v>
       </c>
     </row>
-    <row r="305" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="305" spans="2:7">
       <c r="B305" s="1">
         <v>52824</v>
       </c>
@@ -6580,7 +6563,7 @@
         <v>5.2320000000000002</v>
       </c>
     </row>
-    <row r="306" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="306" spans="2:7">
       <c r="B306" s="1">
         <v>52916</v>
       </c>
@@ -6600,7 +6583,7 @@
         <v>5.2619999999999996</v>
       </c>
     </row>
-    <row r="307" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="307" spans="2:7">
       <c r="B307" s="1">
         <v>52916</v>
       </c>
@@ -6620,7 +6603,7 @@
         <v>5.2279999999999998</v>
       </c>
     </row>
-    <row r="308" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="308" spans="2:7">
       <c r="B308" s="1">
         <v>53008</v>
       </c>
@@ -6640,7 +6623,7 @@
         <v>5.2809999999999997</v>
       </c>
     </row>
-    <row r="309" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="309" spans="2:7">
       <c r="B309" s="1">
         <v>53008</v>
       </c>
@@ -6660,7 +6643,7 @@
         <v>5.2320000000000002</v>
       </c>
     </row>
-    <row r="310" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="310" spans="2:7">
       <c r="B310" s="1">
         <v>53097</v>
       </c>
@@ -6680,7 +6663,7 @@
         <v>5.2729999999999997</v>
       </c>
     </row>
-    <row r="311" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="311" spans="2:7">
       <c r="B311" s="1">
         <v>53097</v>
       </c>
@@ -6700,7 +6683,7 @@
         <v>5.2320000000000002</v>
       </c>
     </row>
-    <row r="312" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="312" spans="2:7">
       <c r="B312" s="1">
         <v>53189</v>
       </c>
@@ -6720,7 +6703,7 @@
         <v>5.2839999999999998</v>
       </c>
     </row>
-    <row r="313" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="313" spans="2:7">
       <c r="B313" s="1">
         <v>53189</v>
       </c>
@@ -6740,7 +6723,7 @@
         <v>5.2409999999999997</v>
       </c>
     </row>
-    <row r="314" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="314" spans="2:7">
       <c r="B314" s="1">
         <v>53281</v>
       </c>
@@ -6760,7 +6743,7 @@
         <v>5.282</v>
       </c>
     </row>
-    <row r="315" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="315" spans="2:7">
       <c r="B315" s="1">
         <v>53281</v>
       </c>
@@ -6780,7 +6763,7 @@
         <v>5.2480000000000002</v>
       </c>
     </row>
-    <row r="316" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="316" spans="2:7">
       <c r="B316" s="1">
         <v>53373</v>
       </c>
@@ -6800,7 +6783,7 @@
         <v>5.298</v>
       </c>
     </row>
-    <row r="317" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="317" spans="2:7">
       <c r="B317" s="1">
         <v>53373</v>
       </c>
@@ -6820,7 +6803,7 @@
         <v>5.25</v>
       </c>
     </row>
-    <row r="318" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="318" spans="2:7">
       <c r="B318" s="1">
         <v>53462</v>
       </c>
@@ -6840,7 +6823,7 @@
         <v>5.3019999999999996</v>
       </c>
     </row>
-    <row r="319" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="319" spans="2:7">
       <c r="B319" s="1">
         <v>53462</v>
       </c>
@@ -6860,7 +6843,7 @@
         <v>5.2469999999999999</v>
       </c>
     </row>
-    <row r="320" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="320" spans="2:7">
       <c r="B320" s="1">
         <v>53554</v>
       </c>
@@ -6880,7 +6863,7 @@
         <v>5.3109999999999999</v>
       </c>
     </row>
-    <row r="321" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="321" spans="2:7">
       <c r="B321" s="1">
         <v>53554</v>
       </c>
@@ -6900,7 +6883,7 @@
         <v>5.2439999999999998</v>
       </c>
     </row>
-    <row r="322" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="322" spans="2:7">
       <c r="B322" s="1">
         <v>53646</v>
       </c>
@@ -6920,7 +6903,7 @@
         <v>5.3010000000000002</v>
       </c>
     </row>
-    <row r="323" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="323" spans="2:7">
       <c r="B323" s="1">
         <v>53738</v>
       </c>
@@ -6940,7 +6923,7 @@
         <v>5.3010000000000002</v>
       </c>
     </row>
-    <row r="324" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="324" spans="2:7">
       <c r="B324" s="1">
         <v>53827</v>
       </c>
@@ -6960,7 +6943,7 @@
         <v>5.3010000000000002</v>
       </c>
     </row>
-    <row r="325" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="325" spans="2:7">
       <c r="B325" s="1">
         <v>53919</v>
       </c>
@@ -6980,7 +6963,7 @@
         <v>5.3120000000000003</v>
       </c>
     </row>
-    <row r="326" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="326" spans="2:7">
       <c r="B326" s="1">
         <v>54011</v>
       </c>
@@ -7000,7 +6983,7 @@
         <v>5.3120000000000003</v>
       </c>
     </row>
-    <row r="327" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="327" spans="2:7">
       <c r="B327" s="1">
         <v>54103</v>
       </c>
@@ -7020,7 +7003,7 @@
         <v>5.3140000000000001</v>
       </c>
     </row>
-    <row r="328" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="328" spans="2:7">
       <c r="B328" s="1">
         <v>54193</v>
       </c>
@@ -7040,7 +7023,7 @@
         <v>5.3109999999999999</v>
       </c>
     </row>
-    <row r="329" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="329" spans="2:7">
       <c r="B329" s="1">
         <v>54285</v>
       </c>
@@ -7060,7 +7043,7 @@
         <v>5.3159999999999998</v>
       </c>
     </row>
-    <row r="330" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="330" spans="2:7">
       <c r="B330" s="1">
         <v>54377</v>
       </c>
@@ -7080,7 +7063,7 @@
         <v>5.3070000000000004</v>
       </c>
     </row>
-    <row r="331" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="331" spans="2:7">
       <c r="B331" s="1">
         <v>54469</v>
       </c>
@@ -7100,7 +7083,7 @@
         <v>5.3150000000000004</v>
       </c>
     </row>
-    <row r="332" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="332" spans="2:7">
       <c r="B332" s="1">
         <v>54558</v>
       </c>
@@ -7120,7 +7103,7 @@
         <v>5.3220000000000001</v>
       </c>
     </row>
-    <row r="333" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="333" spans="2:7">
       <c r="B333" s="1">
         <v>54650</v>
       </c>
@@ -7140,7 +7123,7 @@
         <v>5.3369999999999997</v>
       </c>
     </row>
-    <row r="334" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="334" spans="2:7">
       <c r="B334" s="1">
         <v>54742</v>
       </c>
@@ -7160,7 +7143,7 @@
         <v>5.33</v>
       </c>
     </row>
-    <row r="335" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="335" spans="2:7">
       <c r="B335" s="1">
         <v>54834</v>
       </c>
@@ -7180,7 +7163,7 @@
         <v>5.3369999999999997</v>
       </c>
     </row>
-    <row r="336" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="336" spans="2:7">
       <c r="B336" s="1">
         <v>54923</v>
       </c>
@@ -7200,7 +7183,7 @@
         <v>5.3390000000000004</v>
       </c>
     </row>
-    <row r="337" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="337" spans="2:7">
       <c r="B337" s="1">
         <v>55015</v>
       </c>
@@ -7220,7 +7203,7 @@
         <v>5.3460000000000001</v>
       </c>
     </row>
-    <row r="338" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="338" spans="2:7">
       <c r="B338" s="1">
         <v>55107</v>
       </c>
@@ -7240,7 +7223,7 @@
         <v>5.3460000000000001</v>
       </c>
     </row>
-    <row r="339" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="339" spans="2:7">
       <c r="B339" s="1">
         <v>55199</v>
       </c>
@@ -7260,7 +7243,7 @@
         <v>5.343</v>
       </c>
     </row>
-    <row r="340" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="340" spans="2:7">
       <c r="B340" s="1">
         <v>55288</v>
       </c>
@@ -7280,7 +7263,7 @@
         <v>5.3319999999999999</v>
       </c>
     </row>
-    <row r="341" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="341" spans="2:7">
       <c r="B341" s="1">
         <v>55380</v>
       </c>
@@ -7300,7 +7283,7 @@
         <v>5.3390000000000004</v>
       </c>
     </row>
-    <row r="342" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="342" spans="2:7">
       <c r="B342" s="1">
         <v>55472</v>
       </c>
@@ -7320,7 +7303,7 @@
         <v>5.3369999999999997</v>
       </c>
     </row>
-    <row r="343" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="343" spans="2:7">
       <c r="B343" s="1">
         <v>55564</v>
       </c>
@@ -7340,7 +7323,7 @@
         <v>5.3280000000000003</v>
       </c>
     </row>
-    <row r="344" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="344" spans="2:7">
       <c r="B344" s="1">
         <v>55654</v>
       </c>
@@ -7360,7 +7343,7 @@
         <v>5.3120000000000003</v>
       </c>
     </row>
-    <row r="345" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="345" spans="2:7">
       <c r="B345" s="1">
         <v>55746</v>
       </c>
@@ -7380,7 +7363,7 @@
         <v>5.3109999999999999</v>
       </c>
     </row>
-    <row r="346" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="346" spans="2:7">
       <c r="B346" s="1">
         <v>55838</v>
       </c>
@@ -7400,7 +7383,7 @@
         <v>5.2939999999999996</v>
       </c>
     </row>
-    <row r="347" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="347" spans="2:7">
       <c r="B347" s="1">
         <v>55930</v>
       </c>
@@ -7420,7 +7403,7 @@
         <v>5.2960000000000003</v>
       </c>
     </row>
-    <row r="348" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="348" spans="2:7">
       <c r="B348" s="1">
         <v>56019</v>
       </c>
@@ -7440,7 +7423,7 @@
         <v>5.2939999999999996</v>
       </c>
     </row>
-    <row r="349" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="349" spans="2:7">
       <c r="B349" s="1">
         <v>56111</v>
       </c>
@@ -7460,7 +7443,7 @@
         <v>5.2850000000000001</v>
       </c>
     </row>
-    <row r="350" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="350" spans="2:7">
       <c r="B350" s="1">
         <v>56203</v>
       </c>
@@ -7480,7 +7463,7 @@
         <v>5.2750000000000004</v>
       </c>
     </row>
-    <row r="351" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="351" spans="2:7">
       <c r="B351" s="1">
         <v>56295</v>
       </c>
@@ -7500,7 +7483,7 @@
         <v>5.2789999999999999</v>
       </c>
     </row>
-    <row r="352" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="352" spans="2:7">
       <c r="B352" s="1">
         <v>56384</v>
       </c>
@@ -7520,7 +7503,7 @@
         <v>5.2690000000000001</v>
       </c>
     </row>
-    <row r="353" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="353" spans="2:7">
       <c r="B353" s="1">
         <v>56476</v>
       </c>
@@ -7540,7 +7523,7 @@
         <v>5.2720000000000002</v>
       </c>
     </row>
-    <row r="354" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="354" spans="2:7">
       <c r="B354" s="1">
         <v>56568</v>
       </c>
@@ -7560,7 +7543,7 @@
         <v>5.2670000000000003</v>
       </c>
     </row>
-    <row r="355" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="355" spans="2:7">
       <c r="B355" s="1">
         <v>56660</v>
       </c>
@@ -7580,7 +7563,7 @@
         <v>5.2610000000000001</v>
       </c>
     </row>
-    <row r="356" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="356" spans="2:7">
       <c r="B356" s="1">
         <v>56749</v>
       </c>
@@ -7600,7 +7583,7 @@
         <v>5.2590000000000003</v>
       </c>
     </row>
-    <row r="357" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="357" spans="2:7">
       <c r="B357" s="1">
         <v>56841</v>
       </c>
@@ -7620,7 +7603,7 @@
         <v>5.258</v>
       </c>
     </row>
-    <row r="358" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="358" spans="2:7">
       <c r="B358" s="1">
         <v>56933</v>
       </c>
@@ -7640,7 +7623,7 @@
         <v>5.2549999999999999</v>
       </c>
     </row>
-    <row r="359" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="359" spans="2:7">
       <c r="B359" s="1">
         <v>57025</v>
       </c>
@@ -7660,7 +7643,7 @@
         <v>5.2489999999999997</v>
       </c>
     </row>
-    <row r="360" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="360" spans="2:7">
       <c r="B360" s="1">
         <v>57115</v>
       </c>
@@ -7680,7 +7663,7 @@
         <v>5.2439999999999998</v>
       </c>
     </row>
-    <row r="361" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="361" spans="2:7">
       <c r="B361" s="1">
         <v>57207</v>
       </c>
@@ -7700,7 +7683,7 @@
         <v>5.2409999999999997</v>
       </c>
     </row>
-    <row r="362" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="362" spans="2:7">
       <c r="B362" s="5" t="s">
         <v>11</v>
       </c>

</xml_diff>